<commit_message>
feat(masterdata): 재화·꾸밈·레벨 표 5개 — Currency, CosmeticSlot, Cosmetic(더미 품목), EconomyConfig, LevelCurve
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__beans__.xlsx
+++ b/table/Datas/__beans__.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -677,6 +677,86 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>float</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>가격 한 줄</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>currency_id</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>long</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ReasonCap</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>사유별 일일 상한</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>currency_id</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>long</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(masterdata): Price·ReasonCap 빈은 c,l만 — 서버 패키지에 안 생기게
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/table/Datas/__beans__.xlsx
+++ b/table/Datas/__beans__.xlsx
@@ -691,6 +691,11 @@
           <t>가격 한 줄</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>c,l</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>currency_id</t>
@@ -723,6 +728,11 @@
       <c r="G15" t="inlineStr">
         <is>
           <t>사유별 일일 상한</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>c,l</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">

</xml_diff>